<commit_message>
fix: add Excel text wrapping and dynamic row height
</commit_message>
<xml_diff>
--- a/templates/invoice/invoice template.xlsx
+++ b/templates/invoice/invoice template.xlsx
@@ -41,7 +41,7 @@
       <rPr>
         <color theme="1"/>
         <family val="1"/>
-        <sz val="11"/>
+        <sz val="14"/>
         <rFont val="Times New Roman"/>
       </rPr>
       <t xml:space="preserve"> {{INVOICE_DATE}}</t>
@@ -55,7 +55,7 @@
       <rPr>
         <color theme="1"/>
         <family val="1"/>
-        <sz val="11"/>
+        <sz val="14"/>
         <rFont val="Times New Roman"/>
       </rPr>
       <t xml:space="preserve"> {{INVOICE_NO}}</t>
@@ -288,7 +288,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -296,9 +296,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -321,10 +318,10 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -380,9 +377,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -742,248 +736,248 @@
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
     </row>
     <row r="2" ht="29.25" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
     </row>
     <row r="3" ht="50.25" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="6"/>
-      <c r="B3" s="7"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="9" t="s">
+      <c r="A3" s="5"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="10"/>
-      <c r="F3" s="11" t="s">
+      <c r="E3" s="9"/>
+      <c r="F3" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="12"/>
+      <c r="G3" s="11"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="13"/>
-      <c r="B4" s="14"/>
-      <c r="C4" s="15"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="17"/>
-      <c r="F4" s="11" t="s">
+      <c r="A4" s="12"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="G4" s="12"/>
+      <c r="G4" s="11"/>
     </row>
     <row r="5" ht="113.05" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="18"/>
-      <c r="B5" s="19"/>
-      <c r="C5" s="20"/>
-      <c r="D5" s="21"/>
-      <c r="E5" s="22"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
+      <c r="A5" s="17"/>
+      <c r="B5" s="18"/>
+      <c r="C5" s="19"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
     </row>
     <row r="6" ht="26.25" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="23" t="s">
+      <c r="A6" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="24" t="s">
+      <c r="C6" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="23" t="s">
+      <c r="D6" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="23" t="s">
+      <c r="E6" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="23" t="s">
+      <c r="F6" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="G6" s="23" t="s">
+      <c r="G6" s="22" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="7" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="25" t="s">
+      <c r="A7" s="24" t="s">
         <v>12</v>
       </c>
       <c r="B7" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="26" t="s">
+      <c r="C7" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="25" t="s">
+      <c r="D7" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="25" t="s">
+      <c r="E7" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="27" t="s">
+      <c r="F7" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="G7" s="27" t="s">
+      <c r="G7" s="26" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="8" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="25">
+      <c r="A8" s="24">
         <v>2</v>
       </c>
       <c r="B8" s="25"/>
-      <c r="C8" s="26"/>
-      <c r="D8" s="25"/>
-      <c r="E8" s="25"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="27"/>
+      <c r="C8" s="25"/>
+      <c r="D8" s="24"/>
+      <c r="E8" s="24"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
     </row>
     <row r="9" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="25">
+      <c r="A9" s="24">
         <v>3</v>
       </c>
       <c r="B9" s="25"/>
-      <c r="C9" s="26"/>
-      <c r="D9" s="25"/>
-      <c r="E9" s="25"/>
-      <c r="F9" s="27"/>
-      <c r="G9" s="27"/>
+      <c r="C9" s="25"/>
+      <c r="D9" s="24"/>
+      <c r="E9" s="24"/>
+      <c r="F9" s="26"/>
+      <c r="G9" s="26"/>
     </row>
     <row r="10" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="25">
+      <c r="A10" s="24">
         <v>4</v>
       </c>
       <c r="B10" s="25"/>
-      <c r="C10" s="28"/>
-      <c r="D10" s="29"/>
-      <c r="E10" s="29"/>
-      <c r="F10" s="29"/>
-      <c r="G10" s="27"/>
+      <c r="C10" s="27"/>
+      <c r="D10" s="28"/>
+      <c r="E10" s="28"/>
+      <c r="F10" s="28"/>
+      <c r="G10" s="26"/>
     </row>
     <row r="11" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="25">
+      <c r="A11" s="24">
         <v>5</v>
       </c>
       <c r="B11" s="25"/>
-      <c r="C11" s="28"/>
-      <c r="D11" s="29"/>
-      <c r="E11" s="29"/>
-      <c r="F11" s="27"/>
-      <c r="G11" s="27"/>
+      <c r="C11" s="27"/>
+      <c r="D11" s="28"/>
+      <c r="E11" s="28"/>
+      <c r="F11" s="26"/>
+      <c r="G11" s="26"/>
     </row>
     <row r="12" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="25">
+      <c r="A12" s="24">
         <v>6</v>
       </c>
       <c r="B12" s="25"/>
-      <c r="C12" s="26"/>
-      <c r="D12" s="30"/>
-      <c r="E12" s="25"/>
-      <c r="F12" s="27"/>
-      <c r="G12" s="27"/>
+      <c r="C12" s="25"/>
+      <c r="D12" s="29"/>
+      <c r="E12" s="24"/>
+      <c r="F12" s="26"/>
+      <c r="G12" s="26"/>
     </row>
     <row r="13" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="25">
+      <c r="A13" s="24">
         <v>7</v>
       </c>
       <c r="B13" s="25"/>
-      <c r="C13" s="26"/>
-      <c r="D13" s="25"/>
-      <c r="E13" s="25"/>
-      <c r="F13" s="27"/>
-      <c r="G13" s="27"/>
+      <c r="C13" s="25"/>
+      <c r="D13" s="24"/>
+      <c r="E13" s="24"/>
+      <c r="F13" s="26"/>
+      <c r="G13" s="26"/>
     </row>
     <row r="14" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="25">
+      <c r="A14" s="24">
         <v>8</v>
       </c>
       <c r="B14" s="25"/>
-      <c r="C14" s="26"/>
-      <c r="D14" s="25"/>
-      <c r="E14" s="25"/>
-      <c r="F14" s="27"/>
-      <c r="G14" s="27"/>
+      <c r="C14" s="25"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="24"/>
+      <c r="F14" s="26"/>
+      <c r="G14" s="26"/>
     </row>
     <row r="15" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="25">
+      <c r="A15" s="24">
         <v>9</v>
       </c>
       <c r="B15" s="25"/>
-      <c r="C15" s="26"/>
-      <c r="D15" s="25"/>
-      <c r="E15" s="25"/>
-      <c r="F15" s="27"/>
-      <c r="G15" s="27"/>
+      <c r="C15" s="25"/>
+      <c r="D15" s="24"/>
+      <c r="E15" s="24"/>
+      <c r="F15" s="26"/>
+      <c r="G15" s="26"/>
     </row>
     <row r="16" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="25">
+      <c r="A16" s="24">
         <v>10</v>
       </c>
       <c r="B16" s="25"/>
-      <c r="C16" s="26"/>
-      <c r="D16" s="25"/>
-      <c r="E16" s="25"/>
-      <c r="F16" s="27"/>
-      <c r="G16" s="27"/>
+      <c r="C16" s="25"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="26"/>
+      <c r="G16" s="26"/>
     </row>
     <row r="17" ht="23.25" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="31"/>
-      <c r="B17" s="31"/>
-      <c r="C17" s="32"/>
-      <c r="D17" s="32"/>
-      <c r="E17" s="32"/>
-      <c r="F17" s="33" t="s">
+      <c r="A17" s="30"/>
+      <c r="B17" s="30"/>
+      <c r="C17" s="30"/>
+      <c r="D17" s="30"/>
+      <c r="E17" s="30"/>
+      <c r="F17" s="31" t="s">
         <v>19</v>
       </c>
-      <c r="G17" s="34" t="s">
+      <c r="G17" s="32" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="18" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="32"/>
-      <c r="B18" s="32"/>
-      <c r="C18" s="32"/>
-      <c r="D18" s="32"/>
-      <c r="E18" s="32"/>
-      <c r="F18" s="33" t="s">
+      <c r="A18" s="30"/>
+      <c r="B18" s="30"/>
+      <c r="C18" s="30"/>
+      <c r="D18" s="30"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="G18" s="34" t="s">
+      <c r="G18" s="32" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="32"/>
-      <c r="B19" s="32"/>
-      <c r="C19" s="32"/>
-      <c r="D19" s="32"/>
-      <c r="E19" s="32"/>
-      <c r="F19" s="35" t="s">
+      <c r="A19" s="30"/>
+      <c r="B19" s="30"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="30"/>
+      <c r="E19" s="30"/>
+      <c r="F19" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="G19" s="36" t="s">
+      <c r="G19" s="34" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="20" ht="41.25" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="32"/>
-      <c r="B20" s="32"/>
-      <c r="C20" s="32"/>
-      <c r="D20" s="32"/>
-      <c r="E20" s="32"/>
-      <c r="F20" s="37"/>
-      <c r="G20" s="38"/>
+      <c r="A20" s="30"/>
+      <c r="B20" s="30"/>
+      <c r="C20" s="30"/>
+      <c r="D20" s="30"/>
+      <c r="E20" s="30"/>
+      <c r="F20" s="35"/>
+      <c r="G20" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="9">

</xml_diff>

<commit_message>
feat: add delivery i18n and improve invoice document formatting
</commit_message>
<xml_diff>
--- a/templates/invoice/invoice template.xlsx
+++ b/templates/invoice/invoice template.xlsx
@@ -1,16 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51B8D58D-E789-49B4-9781-0FDF4F9B7DA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14914"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14914" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Sheet1'!$A1:$G20</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A1:$G20</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
@@ -39,10 +40,10 @@
     </r>
     <r>
       <rPr>
+        <sz val="14"/>
         <color theme="1"/>
+        <rFont val="Times New Roman"/>
         <family val="1"/>
-        <sz val="14"/>
-        <rFont val="Times New Roman"/>
       </rPr>
       <t xml:space="preserve"> {{INVOICE_DATE}}</t>
     </r>
@@ -53,10 +54,10 @@
     </r>
     <r>
       <rPr>
+        <sz val="14"/>
         <color theme="1"/>
+        <rFont val="Times New Roman"/>
         <family val="1"/>
-        <sz val="14"/>
-        <rFont val="Times New Roman"/>
       </rPr>
       <t xml:space="preserve"> {{INVOICE_NO}}</t>
     </r>
@@ -125,63 +126,63 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="_ * #,##0.00_ ;_ * -#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
       <charset val="134"/>
-      <color theme="1"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="等线"/>
     </font>
     <font>
       <b/>
+      <sz val="14"/>
       <color theme="1"/>
+      <name val="Times New Roman"/>
       <family val="1"/>
-      <sz val="14"/>
-      <name val="Times New Roman"/>
     </font>
     <font>
       <b/>
+      <sz val="18"/>
       <color theme="1"/>
+      <name val="Times New Roman"/>
       <family val="1"/>
-      <sz val="18"/>
-      <name val="Times New Roman"/>
     </font>
     <font>
+      <sz val="18"/>
       <color theme="1"/>
+      <name val="Times New Roman"/>
       <family val="1"/>
-      <sz val="18"/>
-      <name val="Times New Roman"/>
     </font>
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Times New Roman"/>
       <family val="1"/>
-      <sz val="11"/>
-      <name val="Times New Roman"/>
     </font>
     <font>
+      <sz val="14"/>
       <color theme="1"/>
+      <name val="Times New Roman"/>
       <family val="1"/>
-      <sz val="14"/>
-      <name val="Times New Roman"/>
     </font>
     <font>
+      <sz val="9"/>
+      <name val="等线"/>
+      <family val="3"/>
       <charset val="134"/>
-      <color theme="1"/>
       <scheme val="minor"/>
-      <sz val="14"/>
-      <name val="等线"/>
     </font>
   </fonts>
   <fills count="2">
@@ -192,7 +193,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -201,35 +202,55 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
       <right/>
-      <top style="thin"/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
       <left/>
       <right/>
-      <top style="thin"/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
       <left/>
-      <right style="thin"/>
-      <top style="thin"/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
       <right/>
       <top/>
       <bottom/>
@@ -237,63 +258,97 @@
     </border>
     <border>
       <left/>
-      <right style="thin"/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
       <right/>
       <top/>
-      <bottom style="thin"/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
       <right/>
       <top/>
-      <bottom style="thin"/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
-      <right style="thin"/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top/>
-      <bottom style="thin"/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="43" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -311,90 +366,66 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="6" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="6" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -426,7 +457,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="Picture 1">
+        <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
@@ -715,12 +746,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G20"/>
-  <sheetFormatPr defaultRowHeight="14.15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" defaultColWidth="9" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.15" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.640625" customWidth="1"/>
     <col min="2" max="2" width="13.5" customWidth="1"/>
@@ -731,268 +762,269 @@
     <col min="7" max="7" width="18.640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="99.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:7" ht="99.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-    </row>
-    <row r="2" ht="29.25" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+    </row>
+    <row r="2" spans="1:7" ht="29.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-    </row>
-    <row r="3" ht="50.25" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="5"/>
-      <c r="B3" s="6"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="8" t="s">
+      <c r="B2" s="10"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+    </row>
+    <row r="3" spans="1:7" ht="50.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="12"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="9"/>
-      <c r="F3" s="10" t="s">
+      <c r="E3" s="22"/>
+      <c r="F3" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="11"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="12"/>
-      <c r="B4" s="13"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="15"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="10" t="s">
+      <c r="G3" s="28"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" s="15"/>
+      <c r="B4" s="16"/>
+      <c r="C4" s="17"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="G4" s="11"/>
-    </row>
-    <row r="5" ht="113.05" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="17"/>
-      <c r="B5" s="18"/>
-      <c r="C5" s="19"/>
-      <c r="D5" s="20"/>
-      <c r="E5" s="21"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-    </row>
-    <row r="6" ht="26.25" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="22" t="s">
+      <c r="G4" s="28"/>
+    </row>
+    <row r="5" spans="1:7" ht="113.05" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="18"/>
+      <c r="B5" s="19"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="25"/>
+      <c r="E5" s="26"/>
+      <c r="F5" s="28"/>
+      <c r="G5" s="28"/>
+    </row>
+    <row r="6" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="23" t="s">
+      <c r="B6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="23" t="s">
+      <c r="C6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="22" t="s">
+      <c r="D6" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="22" t="s">
+      <c r="E6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="22" t="s">
+      <c r="F6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="G6" s="22" t="s">
+      <c r="G6" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="24" t="s">
+    <row r="7" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="25" t="s">
+      <c r="B7" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="25" t="s">
+      <c r="C7" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="24" t="s">
+      <c r="D7" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="24" t="s">
+      <c r="E7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="26" t="s">
+      <c r="F7" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="G7" s="26" t="s">
+      <c r="G7" s="6" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="8" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="24">
+    <row r="8" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="4">
         <v>2</v>
       </c>
-      <c r="B8" s="25"/>
-      <c r="C8" s="25"/>
-      <c r="D8" s="24"/>
-      <c r="E8" s="24"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26"/>
-    </row>
-    <row r="9" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="24">
+      <c r="B8" s="5"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="6"/>
+    </row>
+    <row r="9" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="4">
         <v>3</v>
       </c>
-      <c r="B9" s="25"/>
-      <c r="C9" s="25"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="24"/>
-      <c r="F9" s="26"/>
-      <c r="G9" s="26"/>
-    </row>
-    <row r="10" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="24">
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
+    </row>
+    <row r="10" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="4">
         <v>4</v>
       </c>
-      <c r="B10" s="25"/>
-      <c r="C10" s="27"/>
-      <c r="D10" s="28"/>
-      <c r="E10" s="28"/>
-      <c r="F10" s="28"/>
-      <c r="G10" s="26"/>
-    </row>
-    <row r="11" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="24">
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
+    </row>
+    <row r="11" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="4">
         <v>5</v>
       </c>
-      <c r="B11" s="25"/>
-      <c r="C11" s="27"/>
-      <c r="D11" s="28"/>
-      <c r="E11" s="28"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="26"/>
-    </row>
-    <row r="12" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="24">
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
+    </row>
+    <row r="12" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="4">
         <v>6</v>
       </c>
-      <c r="B12" s="25"/>
-      <c r="C12" s="25"/>
-      <c r="D12" s="29"/>
-      <c r="E12" s="24"/>
-      <c r="F12" s="26"/>
-      <c r="G12" s="26"/>
-    </row>
-    <row r="13" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="24">
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
+    </row>
+    <row r="13" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="4">
         <v>7</v>
       </c>
-      <c r="B13" s="25"/>
-      <c r="C13" s="25"/>
-      <c r="D13" s="24"/>
-      <c r="E13" s="24"/>
-      <c r="F13" s="26"/>
-      <c r="G13" s="26"/>
-    </row>
-    <row r="14" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="24">
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
+    </row>
+    <row r="14" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="4">
         <v>8</v>
       </c>
-      <c r="B14" s="25"/>
-      <c r="C14" s="25"/>
-      <c r="D14" s="24"/>
-      <c r="E14" s="24"/>
-      <c r="F14" s="26"/>
-      <c r="G14" s="26"/>
-    </row>
-    <row r="15" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="24">
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="6"/>
+    </row>
+    <row r="15" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="4">
         <v>9</v>
       </c>
-      <c r="B15" s="25"/>
-      <c r="C15" s="25"/>
-      <c r="D15" s="24"/>
-      <c r="E15" s="24"/>
-      <c r="F15" s="26"/>
-      <c r="G15" s="26"/>
-    </row>
-    <row r="16" ht="60" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="24">
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="6"/>
+      <c r="G15" s="6"/>
+    </row>
+    <row r="16" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="4">
         <v>10</v>
       </c>
-      <c r="B16" s="25"/>
-      <c r="C16" s="25"/>
-      <c r="D16" s="24"/>
-      <c r="E16" s="24"/>
-      <c r="F16" s="26"/>
-      <c r="G16" s="26"/>
-    </row>
-    <row r="17" ht="23.25" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="30"/>
-      <c r="B17" s="30"/>
-      <c r="C17" s="30"/>
-      <c r="D17" s="30"/>
-      <c r="E17" s="30"/>
-      <c r="F17" s="31" t="s">
+      <c r="B16" s="5"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="6"/>
+    </row>
+    <row r="17" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A17" s="29"/>
+      <c r="B17" s="29"/>
+      <c r="C17" s="29"/>
+      <c r="D17" s="29"/>
+      <c r="E17" s="29"/>
+      <c r="F17" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="G17" s="32" t="s">
+      <c r="G17" s="8" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="18" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="30"/>
-      <c r="B18" s="30"/>
-      <c r="C18" s="30"/>
-      <c r="D18" s="30"/>
-      <c r="E18" s="30"/>
-      <c r="F18" s="31" t="s">
+    <row r="18" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A18" s="29"/>
+      <c r="B18" s="29"/>
+      <c r="C18" s="29"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="29"/>
+      <c r="F18" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="G18" s="32" t="s">
+      <c r="G18" s="8" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="30"/>
-      <c r="B19" s="30"/>
-      <c r="C19" s="30"/>
-      <c r="D19" s="30"/>
-      <c r="E19" s="30"/>
-      <c r="F19" s="33" t="s">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A19" s="29"/>
+      <c r="B19" s="29"/>
+      <c r="C19" s="29"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="G19" s="34" t="s">
+      <c r="G19" s="32" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="20" ht="41.25" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="30"/>
-      <c r="B20" s="30"/>
-      <c r="C20" s="30"/>
-      <c r="D20" s="30"/>
-      <c r="E20" s="30"/>
-      <c r="F20" s="35"/>
-      <c r="G20" s="36"/>
+    <row r="20" spans="1:7" ht="41.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="29"/>
+      <c r="B20" s="29"/>
+      <c r="C20" s="29"/>
+      <c r="D20" s="29"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="31"/>
+      <c r="G20" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="A17:E20"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="G19:G20"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A3:C5"/>
     <mergeCell ref="D3:E5"/>
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="F4:G5"/>
-    <mergeCell ref="A17:E20"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="G19:G20"/>
   </mergeCells>
-  <pageMargins left="0.699305555555556" right="0.699305555555556" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="67" fitToWidth="1" fitToHeight="0" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
-  <drawing r:id="rId1"/>
+  <phoneticPr fontId="7" type="noConversion"/>
+  <pageMargins left="0.69930555555555596" right="0.69930555555555596" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="59" fitToHeight="0" orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>